<commit_message>
Update APS project command reference
</commit_message>
<xml_diff>
--- a/Commands.xlsx
+++ b/Commands.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Book-Generator\Automated-Processing-System\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F6F745-B577-4DFD-96BB-277301EC05DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,11 +24,149 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+  <si>
+    <t>Commands</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>To check python version</t>
+  </si>
+  <si>
+    <t>py --list</t>
+  </si>
+  <si>
+    <t>Command Prompt (Administrator)</t>
+  </si>
+  <si>
+    <t>py -3.13 -m venv .venv</t>
+  </si>
+  <si>
+    <t>to create python environment</t>
+  </si>
+  <si>
+    <t>to activate python environment</t>
+  </si>
+  <si>
+    <t>.venv\Scripts\activate</t>
+  </si>
+  <si>
+    <t>to upgrade pip</t>
+  </si>
+  <si>
+    <t>python -m pip install --upgrade pip</t>
+  </si>
+  <si>
+    <t>to install add on python</t>
+  </si>
+  <si>
+    <t>pip install -r requirements.txt</t>
+  </si>
+  <si>
+    <t>Github updation</t>
+  </si>
+  <si>
+    <t>git init</t>
+  </si>
+  <si>
+    <t>git add .</t>
+  </si>
+  <si>
+    <t>git commit -m "APS-001A Foundation"</t>
+  </si>
+  <si>
+    <t>to run any python file</t>
+  </si>
+  <si>
+    <t>python main.py</t>
+  </si>
+  <si>
+    <t>git push</t>
+  </si>
+  <si>
+    <t>to set the location</t>
+  </si>
+  <si>
+    <t>Set-Location C:\Automated-Processing-System</t>
+  </si>
+  <si>
+    <t>to create DataBase</t>
+  </si>
+  <si>
+    <t>python -c "import sqlite3; db=sqlite3.connect('database/aps.db'); print('\n'.join(row[0] for row in db.execute(\"SELECT name FROM sqlite_master WHERE type='table' ORDER BY name\"))); db.close()"</t>
+  </si>
+  <si>
+    <t>to verify Database schema</t>
+  </si>
+  <si>
+    <t>git remote -v</t>
+  </si>
+  <si>
+    <t>to check git remote result should be blank if no remote</t>
+  </si>
+  <si>
+    <t>git branch --show-current</t>
+  </si>
+  <si>
+    <t>to set github repository</t>
+  </si>
+  <si>
+    <t>git remote add origin https://github.com/YOUR-USERNAME/Automated-Processing-System.git</t>
+  </si>
+  <si>
+    <t>to check git branch (master / main)</t>
+  </si>
+  <si>
+    <t>git push -u origin main</t>
+  </si>
+  <si>
+    <t>git push -u origin master</t>
+  </si>
+  <si>
+    <t>to update branch if main</t>
+  </si>
+  <si>
+    <t>to update branch if master</t>
+  </si>
+  <si>
+    <t>git remote set-url origin https://github.com/kamranazhar-cmyk/Automated-Processing-System.git</t>
+  </si>
+  <si>
+    <t>Esc</t>
+  </si>
+  <si>
+    <t>To go out git editor</t>
+  </si>
+  <si>
+    <t>:q!</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +181,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -45,12 +189,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +519,802 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="C3:D178"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="50.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="128.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:4" ht="21" x14ac:dyDescent="0.35">
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C17" s="1"/>
+      <c r="D17" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C18" s="1"/>
+      <c r="D18" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C22" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C25" s="4"/>
+      <c r="D25" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C27" s="1"/>
+      <c r="D27" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+    </row>
+    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+    </row>
+    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+    </row>
+    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+    </row>
+    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+    </row>
+    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+    </row>
+    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+    </row>
+    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+    </row>
+    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+    </row>
+    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+    </row>
+    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+    </row>
+    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+    </row>
+    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+    </row>
+    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+    </row>
+    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+    </row>
+    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+    </row>
+    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+    </row>
+    <row r="56" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+    </row>
+    <row r="57" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+    </row>
+    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+    </row>
+    <row r="59" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+    </row>
+    <row r="60" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+    </row>
+    <row r="61" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+    </row>
+    <row r="62" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+    </row>
+    <row r="63" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+    </row>
+    <row r="64" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+    </row>
+    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+    </row>
+    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+    </row>
+    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+    </row>
+    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+    </row>
+    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+    </row>
+    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+    </row>
+    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+    </row>
+    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+    </row>
+    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+    </row>
+    <row r="75" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+    </row>
+    <row r="76" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+    </row>
+    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+    </row>
+    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C78" s="1"/>
+      <c r="D78" s="1"/>
+    </row>
+    <row r="79" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C79" s="1"/>
+      <c r="D79" s="1"/>
+    </row>
+    <row r="80" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C80" s="1"/>
+      <c r="D80" s="1"/>
+    </row>
+    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C81" s="1"/>
+      <c r="D81" s="1"/>
+    </row>
+    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+    </row>
+    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+    </row>
+    <row r="84" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+    </row>
+    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+    </row>
+    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+    </row>
+    <row r="87" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+    </row>
+    <row r="88" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+    </row>
+    <row r="89" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+    </row>
+    <row r="90" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+    </row>
+    <row r="91" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+    </row>
+    <row r="92" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+    </row>
+    <row r="93" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+    </row>
+    <row r="94" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+    </row>
+    <row r="95" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+    </row>
+    <row r="96" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+    </row>
+    <row r="97" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+    </row>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+    </row>
+    <row r="99" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+    </row>
+    <row r="100" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+    </row>
+    <row r="101" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+    </row>
+    <row r="102" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+    </row>
+    <row r="103" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C103" s="1"/>
+      <c r="D103" s="1"/>
+    </row>
+    <row r="104" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+    </row>
+    <row r="105" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
+    </row>
+    <row r="106" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+    </row>
+    <row r="107" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="1"/>
+      <c r="D107" s="1"/>
+    </row>
+    <row r="108" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="1"/>
+      <c r="D108" s="1"/>
+    </row>
+    <row r="109" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C109" s="1"/>
+      <c r="D109" s="1"/>
+    </row>
+    <row r="110" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+    </row>
+    <row r="111" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C111" s="1"/>
+      <c r="D111" s="1"/>
+    </row>
+    <row r="112" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+    </row>
+    <row r="113" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C113" s="1"/>
+      <c r="D113" s="1"/>
+    </row>
+    <row r="114" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+    </row>
+    <row r="115" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C115" s="1"/>
+      <c r="D115" s="1"/>
+    </row>
+    <row r="116" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C116" s="1"/>
+      <c r="D116" s="1"/>
+    </row>
+    <row r="117" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+    </row>
+    <row r="118" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C118" s="1"/>
+      <c r="D118" s="1"/>
+    </row>
+    <row r="119" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+    </row>
+    <row r="120" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C120" s="1"/>
+      <c r="D120" s="1"/>
+    </row>
+    <row r="121" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C121" s="1"/>
+      <c r="D121" s="1"/>
+    </row>
+    <row r="122" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+    </row>
+    <row r="123" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C123" s="1"/>
+      <c r="D123" s="1"/>
+    </row>
+    <row r="124" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C124" s="1"/>
+      <c r="D124" s="1"/>
+    </row>
+    <row r="125" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C125" s="1"/>
+      <c r="D125" s="1"/>
+    </row>
+    <row r="126" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+    </row>
+    <row r="127" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C127" s="1"/>
+      <c r="D127" s="1"/>
+    </row>
+    <row r="128" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C128" s="1"/>
+      <c r="D128" s="1"/>
+    </row>
+    <row r="129" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+    </row>
+    <row r="130" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C130" s="1"/>
+      <c r="D130" s="1"/>
+    </row>
+    <row r="131" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C131" s="1"/>
+      <c r="D131" s="1"/>
+    </row>
+    <row r="132" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C132" s="1"/>
+      <c r="D132" s="1"/>
+    </row>
+    <row r="133" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C133" s="1"/>
+      <c r="D133" s="1"/>
+    </row>
+    <row r="134" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C134" s="1"/>
+      <c r="D134" s="1"/>
+    </row>
+    <row r="135" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C135" s="1"/>
+      <c r="D135" s="1"/>
+    </row>
+    <row r="136" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C136" s="1"/>
+      <c r="D136" s="1"/>
+    </row>
+    <row r="137" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C137" s="1"/>
+      <c r="D137" s="1"/>
+    </row>
+    <row r="138" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C138" s="1"/>
+      <c r="D138" s="1"/>
+    </row>
+    <row r="139" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C139" s="1"/>
+      <c r="D139" s="1"/>
+    </row>
+    <row r="140" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C140" s="1"/>
+      <c r="D140" s="1"/>
+    </row>
+    <row r="141" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C141" s="1"/>
+      <c r="D141" s="1"/>
+    </row>
+    <row r="142" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C142" s="1"/>
+      <c r="D142" s="1"/>
+    </row>
+    <row r="143" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C143" s="1"/>
+      <c r="D143" s="1"/>
+    </row>
+    <row r="144" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C144" s="1"/>
+      <c r="D144" s="1"/>
+    </row>
+    <row r="145" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C145" s="1"/>
+      <c r="D145" s="1"/>
+    </row>
+    <row r="146" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C146" s="1"/>
+      <c r="D146" s="1"/>
+    </row>
+    <row r="147" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C147" s="1"/>
+      <c r="D147" s="1"/>
+    </row>
+    <row r="148" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C148" s="1"/>
+      <c r="D148" s="1"/>
+    </row>
+    <row r="149" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C149" s="1"/>
+      <c r="D149" s="1"/>
+    </row>
+    <row r="150" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C150" s="1"/>
+      <c r="D150" s="1"/>
+    </row>
+    <row r="151" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C151" s="1"/>
+      <c r="D151" s="1"/>
+    </row>
+    <row r="152" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C152" s="1"/>
+      <c r="D152" s="1"/>
+    </row>
+    <row r="153" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C153" s="1"/>
+      <c r="D153" s="1"/>
+    </row>
+    <row r="154" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C154" s="1"/>
+      <c r="D154" s="1"/>
+    </row>
+    <row r="155" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C155" s="1"/>
+      <c r="D155" s="1"/>
+    </row>
+    <row r="156" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C156" s="1"/>
+      <c r="D156" s="1"/>
+    </row>
+    <row r="157" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C157" s="1"/>
+      <c r="D157" s="1"/>
+    </row>
+    <row r="158" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C158" s="1"/>
+      <c r="D158" s="1"/>
+    </row>
+    <row r="159" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C159" s="1"/>
+      <c r="D159" s="1"/>
+    </row>
+    <row r="160" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C160" s="1"/>
+      <c r="D160" s="1"/>
+    </row>
+    <row r="161" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C161" s="1"/>
+      <c r="D161" s="1"/>
+    </row>
+    <row r="162" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C162" s="1"/>
+      <c r="D162" s="1"/>
+    </row>
+    <row r="163" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C163" s="1"/>
+      <c r="D163" s="1"/>
+    </row>
+    <row r="164" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C164" s="1"/>
+      <c r="D164" s="1"/>
+    </row>
+    <row r="165" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C165" s="1"/>
+      <c r="D165" s="1"/>
+    </row>
+    <row r="166" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C166" s="1"/>
+      <c r="D166" s="1"/>
+    </row>
+    <row r="167" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C167" s="1"/>
+      <c r="D167" s="1"/>
+    </row>
+    <row r="168" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C168" s="1"/>
+      <c r="D168" s="1"/>
+    </row>
+    <row r="169" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C169" s="1"/>
+      <c r="D169" s="1"/>
+    </row>
+    <row r="170" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C170" s="1"/>
+      <c r="D170" s="1"/>
+    </row>
+    <row r="171" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C171" s="1"/>
+      <c r="D171" s="1"/>
+    </row>
+    <row r="172" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C172" s="1"/>
+      <c r="D172" s="1"/>
+    </row>
+    <row r="173" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C173" s="1"/>
+      <c r="D173" s="1"/>
+    </row>
+    <row r="174" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C174" s="1"/>
+      <c r="D174" s="1"/>
+    </row>
+    <row r="175" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C175" s="1"/>
+      <c r="D175" s="1"/>
+    </row>
+    <row r="176" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C176" s="1"/>
+      <c r="D176" s="1"/>
+    </row>
+    <row r="177" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C177" s="1"/>
+      <c r="D177" s="1"/>
+    </row>
+    <row r="178" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C178" s="1"/>
+      <c r="D178" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:D3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>